<commit_message>
feat: agrega config central de validacion con todos los validadores CBAM
</commit_message>
<xml_diff>
--- a/tests/fixtures/sample_data.xlsx
+++ b/tests/fixtures/sample_data.xlsx
@@ -566,7 +566,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Complex</t>
+          <t>Complex Goods</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -614,7 +614,6 @@
           <t>Main Street 1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>DEHSt</t>
@@ -625,14 +624,11 @@
           <t>CBAM-DE-2026-00143</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>72071114</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>Iron and Steel</t>
@@ -640,7 +636,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Simple Goods</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -656,13 +652,11 @@
           <t>India</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr">
         <is>
           <t>Supplier In1</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>